<commit_message>
V1.1-last Kicad v7 version
</commit_message>
<xml_diff>
--- a/homebrew_cpu_BOM.xlsx
+++ b/homebrew_cpu_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\prj\yt\ian_ward\homebrew_cpu\Homebrew-CPU-PCB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E0E0F39-45F8-4E0D-9AE5-1EE337C88CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973327D0-9270-4139-879C-48B6FBE8FF84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="13952" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cpu" sheetId="2" r:id="rId1"/>
@@ -95,9 +95,6 @@
     <t>LCD 2004 Female Header</t>
   </si>
   <si>
-    <t>footprints:LCD_2004_PinSocket_1x16_P2.54mm_Vertical</t>
-  </si>
-  <si>
     <t>J2</t>
   </si>
   <si>
@@ -122,30 +119,18 @@
     <t>RN1, RN2, RN3</t>
   </si>
   <si>
-    <t>footprints:R_Array_SIP11</t>
-  </si>
-  <si>
     <t>RV1</t>
   </si>
   <si>
-    <t>footprints:10K_Audio_Slide_Pot</t>
-  </si>
-  <si>
     <t>RV2, RV3</t>
   </si>
   <si>
-    <t>footprints:BOURNE-3386P</t>
-  </si>
-  <si>
     <t>S1</t>
   </si>
   <si>
     <t>RESET</t>
   </si>
   <si>
-    <t>footprints:SW_1825967-1</t>
-  </si>
-  <si>
     <t>S2</t>
   </si>
   <si>
@@ -158,45 +143,30 @@
     <t>TL2230</t>
   </si>
   <si>
-    <t>footprints:TL2230EEF140</t>
-  </si>
-  <si>
     <t>U1, U3</t>
   </si>
   <si>
     <t>LM555</t>
   </si>
   <si>
-    <t>footprints:DIP-8_W7.62mm_Socket</t>
-  </si>
-  <si>
     <t>U2</t>
   </si>
   <si>
     <t>74LS00</t>
   </si>
   <si>
-    <t>footprints:DIP-14_W7.62mm_Socket</t>
-  </si>
-  <si>
     <t>U4, U5, U6, U7, U8</t>
   </si>
   <si>
     <t>74LS163</t>
   </si>
   <si>
-    <t>footprints:DIP-16_W7.62mm_Socket</t>
-  </si>
-  <si>
     <t>U9, U10</t>
   </si>
   <si>
     <t>SST39SF040-70-4C-PHE</t>
   </si>
   <si>
-    <t>footprints:PDIP32_PH_SST_MCH</t>
-  </si>
-  <si>
     <t>Datasheet</t>
   </si>
   <si>
@@ -218,12 +188,6 @@
     <t>D6</t>
   </si>
   <si>
-    <t>footprints:LED_Bar_Graph_10_SEG (Blue)</t>
-  </si>
-  <si>
-    <t>footprints:LED_Bar_Graph_10_SEG (Yellow)</t>
-  </si>
-  <si>
     <t>CUI_UJC-HP-M-G-5-MSMT-TR</t>
   </si>
   <si>
@@ -242,9 +206,6 @@
     <t>3386P-1-502LF</t>
   </si>
   <si>
-    <t>footprints:CUI_UJC-HP-M-G-5-MSMT-TR</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/bourns-inc/4609X-101-471LF/3593678</t>
   </si>
   <si>
@@ -471,6 +432,45 @@
   </si>
   <si>
     <t>Electrolytic capacitor</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:LED_Bar_Graph_10_SEG (Blue)</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:LED_Bar_Graph_10_SEG (Yellow)</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:LCD_2004_PinSocket_1x16_P2.54mm_Vertical</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:CUI_UJC-HP-M-G-5-MSMT-TR</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:R_Array_SIP11</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:10K_Audio_Slide_Pot</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:BOURNE-3386P</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:SW_1825967-1</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:TL2230EEF140</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:DIP-8_W7.62mm_Socket</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:DIP-14_W7.62mm_Socket</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:DIP-16_W7.62mm_Socket</t>
+  </si>
+  <si>
+    <t>Homebrew-CPU-PCB:PDIP32_PH_SST_MCH</t>
   </si>
 </sst>
 </file>
@@ -992,7 +992,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1008,7 +1008,6 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1386,21 +1385,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15C382D7-551C-4DB5-967D-4304CEB98B2E}">
   <dimension ref="A1:I26"/>
-  <sheetFormatPr defaultRowHeight="13.6" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="5"/>
-    <col min="2" max="2" width="19.5" style="2" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" style="2" customWidth="1"/>
     <col min="3" max="3" width="9" style="5"/>
-    <col min="4" max="4" width="25.875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="60.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.75" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="112.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="117.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.85546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="60.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="112.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="117.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="47" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1417,16 +1416,16 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -1440,18 +1439,16 @@
         <v>3</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
+        <v>74</v>
+      </c>
       <c r="I2" s="6" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -1460,28 +1457,28 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="C3" s="5">
         <v>2</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>7</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>65</v>
+        <v>53</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -1502,10 +1499,10 @@
         <v>10</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1526,10 +1523,10 @@
         <v>10</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>117</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1550,10 +1547,10 @@
         <v>10</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -1562,7 +1559,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="C7" s="5">
         <v>2</v>
@@ -1571,19 +1568,19 @@
         <v>15</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>61</v>
+        <v>133</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -1592,7 +1589,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C8" s="5">
         <v>1</v>
@@ -1601,19 +1598,19 @@
         <v>15</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>62</v>
+        <v>134</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -1634,10 +1631,10 @@
         <v>10</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -1655,13 +1652,13 @@
         <v>19</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>20</v>
+        <v>135</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -1670,28 +1667,28 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C11" s="5">
         <v>1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>69</v>
+        <v>136</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -1700,28 +1697,28 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12" s="5">
         <v>3</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -1730,28 +1727,28 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="5">
         <v>4</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -1760,22 +1757,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C14" s="5">
         <v>1</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -1784,22 +1781,22 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C15" s="5">
         <v>1</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -1808,28 +1805,28 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="5">
         <v>2</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -1838,28 +1835,28 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C17" s="5">
         <v>3</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>29</v>
+        <v>137</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
@@ -1868,28 +1865,28 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C18" s="5">
         <v>1</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>31</v>
+        <v>138</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
@@ -1898,28 +1895,28 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C19" s="5">
         <v>2</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>33</v>
+        <v>139</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
@@ -1928,28 +1925,28 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C20" s="5">
         <v>1</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>36</v>
+        <v>140</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
@@ -1958,28 +1955,28 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C21" s="5">
         <v>1</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>36</v>
+        <v>140</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
@@ -1988,28 +1985,28 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C22" s="5">
         <v>1</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>41</v>
+        <v>141</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
@@ -2018,28 +2015,28 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C23" s="5">
         <v>2</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>44</v>
+        <v>142</v>
       </c>
       <c r="F23" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I23" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -2048,28 +2045,28 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C24" s="5">
         <v>1</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>47</v>
+        <v>143</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
@@ -2078,28 +2075,28 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C25" s="5">
         <v>5</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>50</v>
+        <v>144</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
@@ -2108,28 +2105,28 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="C26" s="5">
         <v>2</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>53</v>
+        <v>145</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>